<commit_message>
Add price-driver scatter, re-solve planner at 2% discounting and sync paper
- plots/plot_price_drivers_14.py: price vs China import share, APAC exports and export offers across the 14 equilibria
- Planner benchmark re-solved at 2% (allocation unchanged, duals shift by at most 1.5 USD/kW); welfare and price figures regenerated
- Notes on price indicators, APAC utilisation and idle Chinese capacity

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/llp_planner/llp_planner_results.xlsx
+++ b/outputs/llp_planner/llp_planner_results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="58">
   <si>
     <t>r</t>
   </si>
@@ -146,6 +146,12 @@
   </si>
   <si>
     <t>terminal_salvage_fraction</t>
+  </si>
+  <si>
+    <t>discount_rate</t>
+  </si>
+  <si>
+    <t>base_year</t>
   </si>
   <si>
     <t>solver</t>
@@ -615,31 +621,31 @@
         <v>931</v>
       </c>
       <c r="D2">
-        <v>-230.9999999246666</v>
+        <v>-230.9999999275631</v>
       </c>
       <c r="E2">
-        <v>-3.957850004113271E-11</v>
+        <v>-9.520523930899691E-11</v>
       </c>
       <c r="F2">
-        <v>46.19999998489374</v>
+        <v>46.19999998541742</v>
       </c>
       <c r="G2">
-        <v>324.0000000323916</v>
+        <v>324.0000000323993</v>
       </c>
       <c r="H2">
-        <v>549.0000000549833</v>
+        <v>549.0000000576732</v>
       </c>
       <c r="I2">
-        <v>162.9999999999986</v>
+        <v>162.9999999999999</v>
       </c>
       <c r="J2">
-        <v>7.897662916354577E-12</v>
+        <v>6.25193227669448E-13</v>
       </c>
       <c r="K2">
-        <v>324.0000000323916</v>
+        <v>324.0000000323993</v>
       </c>
       <c r="L2">
-        <v>549.0000000549833</v>
+        <v>549.0000000576732</v>
       </c>
       <c r="M2">
         <v>931</v>
@@ -648,19 +654,19 @@
         <v>163</v>
       </c>
       <c r="O2">
-        <v>262795.6800168896</v>
+        <v>262795.6800168936</v>
       </c>
       <c r="P2">
-        <v>92647.69644215262</v>
+        <v>92647.69644262349</v>
       </c>
       <c r="Q2">
         <v>2327.5</v>
       </c>
       <c r="R2">
-        <v>-1.978925002056636E-09</v>
+        <v>-4.760261965449845E-09</v>
       </c>
       <c r="S2">
-        <v>839102.4178736948</v>
+        <v>839102.4178713744</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -671,34 +677,34 @@
         <v>26</v>
       </c>
       <c r="C3">
-        <v>700.0000000753334</v>
+        <v>700.0000000724368</v>
       </c>
       <c r="D3">
-        <v>-7.821772538025106E-10</v>
+        <v>-7.056739067839135E-11</v>
       </c>
       <c r="E3">
-        <v>-1.891880325215881E-11</v>
+        <v>-9.294121102705609E-11</v>
       </c>
       <c r="F3">
-        <v>1.375166475083433E-10</v>
+        <v>-7.882773289137783E-11</v>
       </c>
       <c r="G3">
-        <v>350.0000000349928</v>
+        <v>350.0000000349994</v>
       </c>
       <c r="H3">
-        <v>674.0000000631636</v>
+        <v>674.0000000697714</v>
       </c>
       <c r="I3">
-        <v>107.4409237870698</v>
+        <v>107.4409237869827</v>
       </c>
       <c r="J3">
-        <v>1.052723406104195E-10</v>
+        <v>1.032309722518128E-11</v>
       </c>
       <c r="K3">
-        <v>350.0000000349926</v>
+        <v>350.0000000349993</v>
       </c>
       <c r="L3">
-        <v>674.0000000631636</v>
+        <v>674.0000000697714</v>
       </c>
       <c r="M3">
         <v>931</v>
@@ -707,19 +713,19 @@
         <v>107.4409237869731</v>
       </c>
       <c r="O3">
-        <v>283884.2222404681</v>
+        <v>283884.2222404716</v>
       </c>
       <c r="P3">
-        <v>76929.5351354771</v>
+        <v>76929.53513627013</v>
       </c>
       <c r="Q3">
-        <v>1750.000000188334</v>
+        <v>1750.000000181092</v>
       </c>
       <c r="R3">
-        <v>-9.459401626079404E-10</v>
+        <v>-4.647060551352805E-09</v>
       </c>
       <c r="S3">
-        <v>1026023.435524018</v>
+        <v>929301.0371581158</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -730,34 +736,34 @@
         <v>27</v>
       </c>
       <c r="C4">
-        <v>700.0000000745513</v>
+        <v>700.0000000723663</v>
       </c>
       <c r="D4">
-        <v>-3.474998103605036E-11</v>
+        <v>5.075736078460166E-13</v>
       </c>
       <c r="E4">
-        <v>1.737882079921272E-11</v>
+        <v>-8.82594555828352E-11</v>
       </c>
       <c r="F4">
-        <v>2.432881700642279E-11</v>
+        <v>-8.83609703044044E-11</v>
       </c>
       <c r="G4">
-        <v>333.0000000332929</v>
+        <v>333.0000000332993</v>
       </c>
       <c r="H4">
-        <v>700.000000062332</v>
+        <v>700.0000000712608</v>
       </c>
       <c r="I4">
-        <v>96.03096600012995</v>
+        <v>95.81429190391654</v>
       </c>
       <c r="J4">
-        <v>0.4551329997343792</v>
+        <v>0.2384589035127895</v>
       </c>
       <c r="K4">
-        <v>333.0000000332928</v>
+        <v>333.0000000332993</v>
       </c>
       <c r="L4">
-        <v>700.000000062332</v>
+        <v>700.0000000712608</v>
       </c>
       <c r="M4">
         <v>931</v>
@@ -766,19 +772,19 @@
         <v>95.57583300040461</v>
       </c>
       <c r="O4">
-        <v>270095.5600173596</v>
+        <v>270095.5600173629</v>
       </c>
       <c r="P4">
-        <v>71996.10626173414</v>
+        <v>71996.1062626973</v>
       </c>
       <c r="Q4">
-        <v>1750.000000186378</v>
+        <v>1750.000000180916</v>
       </c>
       <c r="R4">
-        <v>8.689410399606359E-10</v>
+        <v>-4.41297277914176E-09</v>
       </c>
       <c r="S4">
-        <v>981747.2687771907</v>
+        <v>805374.7028445528</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -789,34 +795,34 @@
         <v>28</v>
       </c>
       <c r="C5">
-        <v>700.0000000745165</v>
+        <v>700.0000000723668</v>
       </c>
       <c r="D5">
-        <v>5.610504425293956E-13</v>
+        <v>-1.227555001582367E-11</v>
       </c>
       <c r="E5">
-        <v>2.095843823706302E-11</v>
+        <v>-8.820557972591557E-11</v>
       </c>
       <c r="F5">
-        <v>2.084622814855714E-11</v>
+        <v>-8.575046972275084E-11</v>
       </c>
       <c r="G5">
-        <v>316.000000031593</v>
+        <v>316.0000000315993</v>
       </c>
       <c r="H5">
-        <v>700.0000000733511</v>
+        <v>700.000000072375</v>
       </c>
       <c r="I5">
-        <v>88.38012419954521</v>
+        <v>89.85101331051274</v>
       </c>
       <c r="J5">
-        <v>2.044867000143244</v>
+        <v>3.515756111102258</v>
       </c>
       <c r="K5">
-        <v>316.000000031593</v>
+        <v>316.0000000315993</v>
       </c>
       <c r="L5">
-        <v>700.0000000733511</v>
+        <v>700.000000072375</v>
       </c>
       <c r="M5">
         <v>931</v>
@@ -825,19 +831,19 @@
         <v>86.33525719941149</v>
       </c>
       <c r="O5">
-        <v>256306.897794251</v>
+        <v>256306.8977942542</v>
       </c>
       <c r="P5">
-        <v>65740.00050889925</v>
+        <v>65740.00050878404</v>
       </c>
       <c r="Q5">
-        <v>1750.000000186291</v>
+        <v>1750.000000180917</v>
       </c>
       <c r="R5">
-        <v>1.047921911853151E-09</v>
+        <v>-4.410278986295779E-09</v>
       </c>
       <c r="S5">
-        <v>944084.4864258219</v>
+        <v>701468.6797685121</v>
       </c>
     </row>
     <row r="6" spans="1:19">
@@ -851,31 +857,31 @@
         <v>22</v>
       </c>
       <c r="D6">
-        <v>-21.99999999646378</v>
+        <v>-22.00000000004764</v>
       </c>
       <c r="E6">
-        <v>-8.271967023443485E-11</v>
+        <v>-9.863006445777678E-11</v>
       </c>
       <c r="F6">
-        <v>4.399999999210037</v>
+        <v>4.399999999910898</v>
       </c>
       <c r="G6">
-        <v>75.00000000749617</v>
+        <v>75.00000000749971</v>
       </c>
       <c r="H6">
-        <v>-4.669969580750083E-10</v>
+        <v>-5.894481237724103E-10</v>
       </c>
       <c r="I6">
-        <v>179.1179999999677</v>
+        <v>179.1179999999974</v>
       </c>
       <c r="J6">
-        <v>1.369382114307271E-10</v>
+        <v>1.089471389026332E-11</v>
       </c>
       <c r="K6">
-        <v>75.00000000749618</v>
+        <v>75.00000000749971</v>
       </c>
       <c r="L6">
-        <v>-4.669969580750083E-10</v>
+        <v>-5.894481237724103E-10</v>
       </c>
       <c r="M6">
         <v>22</v>
@@ -884,19 +890,19 @@
         <v>299.25</v>
       </c>
       <c r="O6">
-        <v>112892.5000072537</v>
+        <v>112892.5000072571</v>
       </c>
       <c r="P6">
-        <v>-1.453558481228694E-07</v>
+        <v>-1.833967256801488E-07</v>
       </c>
       <c r="Q6">
         <v>192.5</v>
       </c>
       <c r="R6">
-        <v>-1.44759422910261E-08</v>
+        <v>-1.726026128011094E-08</v>
       </c>
       <c r="S6">
-        <v>563500.0000370676</v>
+        <v>563500.0000372888</v>
       </c>
     </row>
     <row r="7" spans="1:19">
@@ -907,34 +913,34 @@
         <v>26</v>
       </c>
       <c r="C7">
-        <v>3.536214493678246E-09</v>
+        <v>-4.76457492537245E-11</v>
       </c>
       <c r="D7">
-        <v>-3.60397126578905E-10</v>
+        <v>-3.279255224787886E-11</v>
       </c>
       <c r="E7">
-        <v>-7.888223865026798E-11</v>
+        <v>-9.8173587497365E-11</v>
       </c>
       <c r="F7">
-        <v>-6.802813334486979E-12</v>
+        <v>-9.161507704778923E-11</v>
       </c>
       <c r="G7">
-        <v>90.00000000899642</v>
+        <v>90.00000000899969</v>
       </c>
       <c r="H7">
-        <v>-3.99181717628836E-10</v>
+        <v>-5.82178688578423E-10</v>
       </c>
       <c r="I7">
-        <v>123.5589237870451</v>
+        <v>123.5589237869805</v>
       </c>
       <c r="J7">
-        <v>0.8061538522957509</v>
+        <v>0.9959412579635974</v>
       </c>
       <c r="K7">
-        <v>90.00000000899644</v>
+        <v>90.00000000899969</v>
       </c>
       <c r="L7">
-        <v>-3.99181717628836E-10</v>
+        <v>-5.82178688578423E-10</v>
       </c>
       <c r="M7">
         <v>22</v>
@@ -943,19 +949,19 @@
         <v>197.2496714309921</v>
       </c>
       <c r="O7">
-        <v>135471.0000087054</v>
+        <v>135471.0000087085</v>
       </c>
       <c r="P7">
-        <v>-8.362202391575218E-08</v>
+        <v>-1.2176061772036E-07</v>
       </c>
       <c r="Q7">
-        <v>3.094187681968465E-08</v>
+        <v>-4.169003059700894E-10</v>
       </c>
       <c r="R7">
-        <v>-1.38043917637969E-08</v>
+        <v>-1.718037781203888E-08</v>
       </c>
       <c r="S7">
-        <v>677355.0000438594</v>
+        <v>613501.2927324118</v>
       </c>
     </row>
     <row r="8" spans="1:19">
@@ -966,34 +972,34 @@
         <v>27</v>
       </c>
       <c r="C8">
-        <v>3.17581736710077E-09</v>
+        <v>-8.043830150162776E-11</v>
       </c>
       <c r="D8">
-        <v>-1.053432987675921E-10</v>
+        <v>-1.059372747761936E-11</v>
       </c>
       <c r="E8">
-        <v>-7.314845192025205E-11</v>
+        <v>-9.744765912042352E-11</v>
       </c>
       <c r="F8">
-        <v>-5.207979216673363E-11</v>
+        <v>-9.532891362489965E-11</v>
       </c>
       <c r="G8">
-        <v>95.00000000949647</v>
+        <v>95.00000000949966</v>
       </c>
       <c r="H8">
-        <v>-3.734845566295888E-10</v>
+        <v>-5.776444370763107E-10</v>
       </c>
       <c r="I8">
-        <v>112.1489660001075</v>
+        <v>111.9322919039143</v>
       </c>
       <c r="J8">
-        <v>0.9209193344460311</v>
+        <v>1.287213618556058</v>
       </c>
       <c r="K8">
-        <v>95.00000000949649</v>
+        <v>95.00000000949966</v>
       </c>
       <c r="L8">
-        <v>-3.734845566295888E-10</v>
+        <v>-5.776444370763107E-10</v>
       </c>
       <c r="M8">
         <v>22</v>
@@ -1002,19 +1008,19 @@
         <v>175.4666750022766</v>
       </c>
       <c r="O8">
-        <v>142997.1666758559</v>
+        <v>142997.166675859</v>
       </c>
       <c r="P8">
-        <v>-7.015300226398679E-08</v>
+        <v>-1.082351923637131E-07</v>
       </c>
       <c r="Q8">
-        <v>2.778840196213174E-08</v>
+        <v>-7.038351381392429E-10</v>
       </c>
       <c r="R8">
-        <v>-1.280097908604411E-08</v>
+        <v>-1.705334034607412E-08</v>
       </c>
       <c r="S8">
-        <v>714985.8333795554</v>
+        <v>586537.4128480424</v>
       </c>
     </row>
     <row r="9" spans="1:19">
@@ -1025,34 +1031,34 @@
         <v>28</v>
       </c>
       <c r="C9">
-        <v>3.070474068332966E-09</v>
+        <v>-9.103202897925457E-11</v>
       </c>
       <c r="D9">
-        <v>2.121182023401106E-11</v>
+        <v>2.545886318290489E-12</v>
       </c>
       <c r="E9">
-        <v>-6.333660326501098E-11</v>
+        <v>-9.610274794351087E-11</v>
       </c>
       <c r="F9">
-        <v>-6.757896731181319E-11</v>
+        <v>-9.661192520716897E-11</v>
       </c>
       <c r="G9">
-        <v>99.00000000989651</v>
+        <v>99.00000000989964</v>
       </c>
       <c r="H9">
-        <v>-3.409496934083979E-10</v>
+        <v>-5.709974551313816E-10</v>
       </c>
       <c r="I9">
-        <v>104.4981241995246</v>
+        <v>105.9690133105105</v>
       </c>
       <c r="J9">
-        <v>0.9579316369230153</v>
+        <v>1.546457072652951</v>
       </c>
       <c r="K9">
-        <v>99.0000000098965</v>
+        <v>99.00000000989961</v>
       </c>
       <c r="L9">
-        <v>-3.409496934083979E-10</v>
+        <v>-5.709974551313816E-10</v>
       </c>
       <c r="M9">
         <v>22</v>
@@ -1061,19 +1067,19 @@
         <v>158.5019982633367</v>
       </c>
       <c r="O9">
-        <v>149018.1000095764</v>
+        <v>149018.1000095794</v>
       </c>
       <c r="P9">
-        <v>-5.833275053604045E-08</v>
+        <v>-9.731321725254296E-08</v>
       </c>
       <c r="Q9">
-        <v>2.686664809791345E-08</v>
+        <v>-7.965302535684774E-10</v>
       </c>
       <c r="R9">
-        <v>-1.108390557137692E-08</v>
+        <v>-1.68179808901144E-08</v>
       </c>
       <c r="S9">
-        <v>745090.5000480945</v>
+        <v>553613.2167105256</v>
       </c>
     </row>
     <row r="10" spans="1:19">
@@ -1087,31 +1093,31 @@
         <v>42</v>
       </c>
       <c r="D10">
-        <v>-41.99999999648314</v>
+        <v>-42.00000000004481</v>
       </c>
       <c r="E10">
-        <v>-8.273179953818707E-11</v>
+        <v>-9.86300674273924E-11</v>
       </c>
       <c r="F10">
-        <v>8.399999999213897</v>
+        <v>8.399999999910332</v>
       </c>
       <c r="G10">
-        <v>45.00000000449219</v>
+        <v>45.00000000449938</v>
       </c>
       <c r="H10">
-        <v>-4.862780123085512E-10</v>
+        <v>-5.909756390966426E-10</v>
       </c>
       <c r="I10">
-        <v>174.132999999941</v>
+        <v>174.1329999999953</v>
       </c>
       <c r="J10">
-        <v>7.180329866366077E-11</v>
+        <v>5.705630722308271E-12</v>
       </c>
       <c r="K10">
-        <v>45.0000000044922</v>
+        <v>45.00000000449938</v>
       </c>
       <c r="L10">
-        <v>-4.862780123085512E-10</v>
+        <v>-5.909756390966426E-10</v>
       </c>
       <c r="M10">
         <v>42</v>
@@ -1120,19 +1126,19 @@
         <v>321.25</v>
       </c>
       <c r="O10">
-        <v>39274.90000252044</v>
+        <v>39274.90000252447</v>
       </c>
       <c r="P10">
-        <v>-1.625520393579331E-07</v>
+        <v>-1.974900792124222E-07</v>
       </c>
       <c r="Q10">
         <v>367.5</v>
       </c>
       <c r="R10">
-        <v>-1.447806491918274E-08</v>
+        <v>-1.726026179979367E-08</v>
       </c>
       <c r="S10">
-        <v>194537.0000134874</v>
+        <v>194537.0000136961</v>
       </c>
     </row>
     <row r="11" spans="1:19">
@@ -1143,34 +1149,34 @@
         <v>26</v>
       </c>
       <c r="C11">
-        <v>3.516851702299031E-09</v>
+        <v>-4.481075861564836E-11</v>
       </c>
       <c r="D11">
-        <v>-3.59554529717896E-10</v>
+        <v>-3.272013259494647E-11</v>
       </c>
       <c r="E11">
-        <v>-7.890370906523213E-11</v>
+        <v>-9.81728938212255E-11</v>
       </c>
       <c r="F11">
-        <v>-6.992803121652925E-12</v>
+        <v>-9.162886730223621E-11</v>
       </c>
       <c r="G11">
-        <v>65.00000000649318</v>
+        <v>65.00000000649941</v>
       </c>
       <c r="H11">
-        <v>-4.288439240962129E-10</v>
+        <v>-5.848380893564396E-10</v>
       </c>
       <c r="I11">
-        <v>118.5739237870321</v>
+        <v>118.5739237869794</v>
       </c>
       <c r="J11">
-        <v>0.8278743206134717</v>
+        <v>0.9881703162601674</v>
       </c>
       <c r="K11">
-        <v>65.00000000649318</v>
+        <v>65.00000000649941</v>
       </c>
       <c r="L11">
-        <v>-4.288439240962129E-10</v>
+        <v>-5.848380893564396E-10</v>
       </c>
       <c r="M11">
         <v>42</v>
@@ -1179,19 +1185,19 @@
         <v>211.7509004083749</v>
       </c>
       <c r="O11">
-        <v>56730.41111475424</v>
+        <v>56730.41111475774</v>
       </c>
       <c r="P11">
-        <v>-9.646569908211818E-08</v>
+        <v>-1.314061516808055E-07</v>
       </c>
       <c r="Q11">
-        <v>3.077245239511652E-08</v>
+        <v>-3.920941378869232E-10</v>
       </c>
       <c r="R11">
-        <v>-1.380814908641562E-08</v>
+        <v>-1.718025641871446E-08</v>
       </c>
       <c r="S11">
-        <v>283652.0555741687</v>
+        <v>256912.4060054426</v>
       </c>
     </row>
     <row r="12" spans="1:19">
@@ -1202,34 +1208,34 @@
         <v>27</v>
       </c>
       <c r="C12">
-        <v>3.157297172587858E-09</v>
+        <v>-7.753089121061054E-11</v>
       </c>
       <c r="D12">
-        <v>-1.053891754547967E-10</v>
+        <v>-1.054863382428637E-11</v>
       </c>
       <c r="E12">
-        <v>-7.318910353797303E-11</v>
+        <v>-9.74460675949802E-11</v>
       </c>
       <c r="F12">
-        <v>-5.21112684470137E-11</v>
+        <v>-9.533634083012293E-11</v>
       </c>
       <c r="G12">
-        <v>70.00000000699335</v>
+        <v>70.00000000699936</v>
       </c>
       <c r="H12">
-        <v>-4.073665122365731E-10</v>
+        <v>-5.810431065339229E-10</v>
       </c>
       <c r="I12">
-        <v>107.1639660000961</v>
+        <v>106.9472919039132</v>
       </c>
       <c r="J12">
-        <v>0.9243117561715705</v>
+        <v>1.272917760163183</v>
       </c>
       <c r="K12">
-        <v>70.00000000699333</v>
+        <v>70.00000000699933</v>
       </c>
       <c r="L12">
-        <v>-4.073665122365731E-10</v>
+        <v>-5.810431065339229E-10</v>
       </c>
       <c r="M12">
         <v>42</v>
@@ -1238,19 +1244,19 @@
         <v>188.3664806833128</v>
       </c>
       <c r="O12">
-        <v>61094.28889281265</v>
+        <v>61094.28889281602</v>
       </c>
       <c r="P12">
-        <v>-8.214452259393545E-08</v>
+        <v>-1.16970415540304E-07</v>
       </c>
       <c r="Q12">
-        <v>2.762635026014376E-08</v>
+        <v>-6.783952980928423E-10</v>
       </c>
       <c r="R12">
-        <v>-1.280809311914528E-08</v>
+        <v>-1.705306182912154E-08</v>
       </c>
       <c r="S12">
-        <v>305471.4444643999</v>
+        <v>250592.9801270685</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -1261,34 +1267,34 @@
         <v>28</v>
       </c>
       <c r="C13">
-        <v>3.051907997126497E-09</v>
+        <v>-8.807952503492338E-11</v>
       </c>
       <c r="D13">
-        <v>2.085252597658635E-11</v>
+        <v>2.534343135649681E-12</v>
       </c>
       <c r="E13">
-        <v>-6.34180276216116E-11</v>
+        <v>-9.610560299789883E-11</v>
       </c>
       <c r="F13">
-        <v>-6.758853281692887E-11</v>
+        <v>-9.661247162502876E-11</v>
       </c>
       <c r="G13">
-        <v>75.00000000749345</v>
+        <v>75.00000000749931</v>
       </c>
       <c r="H13">
-        <v>-3.812176409284717E-10</v>
+        <v>-5.756994897191019E-10</v>
       </c>
       <c r="I13">
-        <v>99.51312419951462</v>
+        <v>100.9840133105094</v>
       </c>
       <c r="J13">
-        <v>0.9645260078928437</v>
+        <v>1.519641915956633</v>
       </c>
       <c r="K13">
-        <v>75.00000000749345</v>
+        <v>75.00000000749931</v>
       </c>
       <c r="L13">
-        <v>-3.812176409284717E-10</v>
+        <v>-5.756994897191019E-10</v>
       </c>
       <c r="M13">
         <v>42</v>
@@ -1297,19 +1303,19 @@
         <v>170.1546096644843</v>
       </c>
       <c r="O13">
-        <v>65458.16667087103</v>
+        <v>65458.16667087431</v>
       </c>
       <c r="P13">
-        <v>-6.997952885290931E-08</v>
+        <v>-1.054172273300571E-07</v>
       </c>
       <c r="Q13">
-        <v>2.670419497485685E-08</v>
+        <v>-7.706958440555796E-10</v>
       </c>
       <c r="R13">
-        <v>-1.109815483378203E-08</v>
+        <v>-1.68184805246323E-08</v>
       </c>
       <c r="S13">
-        <v>327290.833354627</v>
+        <v>243181.9101729727</v>
       </c>
     </row>
     <row r="14" spans="1:19">
@@ -1323,31 +1329,31 @@
         <v>110</v>
       </c>
       <c r="D14">
-        <v>-77.00000000711726</v>
+        <v>-76.99999999762035</v>
       </c>
       <c r="E14">
-        <v>-4.745383424547862E-11</v>
+        <v>-9.583065160417894E-11</v>
       </c>
       <c r="F14">
-        <v>15.400000001376</v>
+        <v>15.39999999942824</v>
       </c>
       <c r="G14">
-        <v>50.00000000499154</v>
+        <v>50.00000000499933</v>
       </c>
       <c r="H14">
-        <v>2.155845226131939E-10</v>
+        <v>-5.353863775590849E-10</v>
       </c>
       <c r="I14">
-        <v>176.7804215788295</v>
+        <v>176.7804215788775</v>
       </c>
       <c r="J14">
-        <v>2.734974681227867E-11</v>
+        <v>2.17702207603463E-12</v>
       </c>
       <c r="K14">
-        <v>50.00000000499154</v>
+        <v>50.00000000499933</v>
       </c>
       <c r="L14">
-        <v>2.155845226131939E-10</v>
+        <v>-5.353863775590849E-10</v>
       </c>
       <c r="M14">
         <v>110</v>
@@ -1356,19 +1362,19 @@
         <v>187.45</v>
       </c>
       <c r="O14">
-        <v>41544.22222488841</v>
+        <v>41544.22222489257</v>
       </c>
       <c r="P14">
-        <v>4.093565863536825E-08</v>
+        <v>-1.072502593121641E-07</v>
       </c>
       <c r="Q14">
         <v>316.25</v>
       </c>
       <c r="R14">
-        <v>-2.728595469115021E-09</v>
+        <v>-5.510262467240289E-09</v>
       </c>
       <c r="S14">
-        <v>206139.861124251</v>
+        <v>206139.8611250266</v>
       </c>
     </row>
     <row r="15" spans="1:19">
@@ -1379,34 +1385,34 @@
         <v>26</v>
       </c>
       <c r="C15">
-        <v>32.99999999288271</v>
+        <v>33.00000000237965</v>
       </c>
       <c r="D15">
-        <v>-6.6669695175094E-10</v>
+        <v>-6.137833309255767E-11</v>
       </c>
       <c r="E15">
-        <v>-2.910228982323429E-11</v>
+        <v>-9.38622534004111E-11</v>
       </c>
       <c r="F15">
-        <v>1.042371005269537E-10</v>
+        <v>-8.158658678189956E-11</v>
       </c>
       <c r="G15">
-        <v>85.00000000849268</v>
+        <v>85.00000000849936</v>
       </c>
       <c r="H15">
-        <v>1.453223321272127E-09</v>
+        <v>-4.202214951496967E-10</v>
       </c>
       <c r="I15">
-        <v>121.2213453659249</v>
+        <v>121.221345365862</v>
       </c>
       <c r="J15">
-        <v>9.526356530428659E-11</v>
+        <v>8.015717492363811E-12</v>
       </c>
       <c r="K15">
-        <v>85.00000000849268</v>
+        <v>85.00000000849936</v>
       </c>
       <c r="L15">
-        <v>1.453223321272127E-09</v>
+        <v>-4.202214951496967E-10</v>
       </c>
       <c r="M15">
         <v>110</v>
@@ -1415,19 +1421,19 @@
         <v>123.5570623550191</v>
       </c>
       <c r="O15">
-        <v>70625.17778231406</v>
+        <v>70625.17778231762</v>
       </c>
       <c r="P15">
-        <v>1.835436684715278E-07</v>
+        <v>-5.844312828005883E-08</v>
       </c>
       <c r="Q15">
-        <v>94.8749999795378</v>
+        <v>94.87500000684149</v>
       </c>
       <c r="R15">
-        <v>-1.673381664835972E-09</v>
+        <v>-5.397079570523638E-09</v>
       </c>
       <c r="S15">
-        <v>352651.5139107633</v>
+        <v>319407.3412831467</v>
       </c>
     </row>
     <row r="16" spans="1:19">
@@ -1438,34 +1444,34 @@
         <v>27</v>
       </c>
       <c r="C16">
-        <v>32.99999999221602</v>
+        <v>33.00000000231827</v>
       </c>
       <c r="D16">
-        <v>3.545964754693147E-11</v>
+        <v>5.304536103120217E-12</v>
       </c>
       <c r="E16">
-        <v>8.893733022702241E-12</v>
+        <v>-8.927705095988832E-11</v>
       </c>
       <c r="F16">
-        <v>1.801803513315947E-12</v>
+        <v>-9.033795818051236E-11</v>
       </c>
       <c r="G16">
-        <v>103.0000000102929</v>
+        <v>103.0000000102993</v>
       </c>
       <c r="H16">
-        <v>1.353335836562902E-09</v>
+        <v>4.027518300778825E-10</v>
       </c>
       <c r="I16">
-        <v>109.811387578993</v>
+        <v>109.5947134827963</v>
       </c>
       <c r="J16">
-        <v>8.213293762164717E-11</v>
+        <v>8.851459650004213E-12</v>
       </c>
       <c r="K16">
-        <v>103.0000000102929</v>
+        <v>103.0000000102993</v>
       </c>
       <c r="L16">
-        <v>1.353335836562902E-09</v>
+        <v>4.027518300778825E-10</v>
       </c>
       <c r="M16">
         <v>110</v>
@@ -1474,19 +1480,19 @@
         <v>109.9122079504653</v>
       </c>
       <c r="O16">
-        <v>85581.09778327563</v>
+        <v>85581.09778327905</v>
       </c>
       <c r="P16">
-        <v>1.54091297398406E-07</v>
+        <v>3.798189999300016E-08</v>
       </c>
       <c r="Q16">
-        <v>94.87499997762106</v>
+        <v>94.87500000666503</v>
       </c>
       <c r="R16">
-        <v>5.113896488053789E-10</v>
+        <v>-5.133430430193578E-09</v>
       </c>
       <c r="S16">
-        <v>427431.1139157171</v>
+        <v>350642.3876148966</v>
       </c>
     </row>
     <row r="17" spans="1:19">
@@ -1497,34 +1503,34 @@
         <v>28</v>
       </c>
       <c r="C17">
-        <v>32.99999999225147</v>
+        <v>33.00000000232357</v>
       </c>
       <c r="D17">
-        <v>-5.165604054341955E-12</v>
+        <v>-1.067428666663233E-11</v>
       </c>
       <c r="E17">
-        <v>4.750972632341401E-12</v>
+        <v>-8.97439468207046E-11</v>
       </c>
       <c r="F17">
-        <v>5.784093443209792E-12</v>
+        <v>-8.760908948737813E-11</v>
       </c>
       <c r="G17">
-        <v>126.000000012593</v>
+        <v>126.0000000125992</v>
       </c>
       <c r="H17">
-        <v>32.9999999914015</v>
+        <v>33.00000000234932</v>
       </c>
       <c r="I17">
-        <v>102.1605457784046</v>
+        <v>103.6314348893919</v>
       </c>
       <c r="J17">
-        <v>2.874999999176164</v>
+        <v>4.345889110078492</v>
       </c>
       <c r="K17">
-        <v>126.000000012593</v>
+        <v>126.0000000125993</v>
       </c>
       <c r="L17">
-        <v>32.9999999914015</v>
+        <v>33.00000000234932</v>
       </c>
       <c r="M17">
         <v>110</v>
@@ -1533,19 +1539,19 @@
         <v>99.28554577932321</v>
       </c>
       <c r="O17">
-        <v>104691.4400067264</v>
+        <v>104691.4400067298</v>
       </c>
       <c r="P17">
-        <v>3276.423009869569</v>
+        <v>3276.42301094479</v>
       </c>
       <c r="Q17">
-        <v>94.87499997772299</v>
+        <v>94.87500000668028</v>
       </c>
       <c r="R17">
-        <v>2.731809263596305E-10</v>
+        <v>-5.160276942190514E-09</v>
       </c>
       <c r="S17">
-        <v>506600.7099843944</v>
+        <v>376411.7897369773</v>
       </c>
     </row>
     <row r="18" spans="1:19">
@@ -1559,31 +1565,31 @@
         <v>3.4</v>
       </c>
       <c r="D18">
-        <v>-3.399999989279363</v>
+        <v>-3.399999999700616</v>
       </c>
       <c r="E18">
-        <v>-7.965506357125596E-11</v>
+        <v>-9.840166494196983E-11</v>
       </c>
       <c r="F18">
-        <v>0.6799999977762174</v>
+        <v>0.6799999998417215</v>
       </c>
       <c r="G18">
-        <v>10.00000000099686</v>
+        <v>10.00000000099975</v>
       </c>
       <c r="H18">
-        <v>1.123714967236795E-09</v>
+        <v>-4.678584044303851E-10</v>
       </c>
       <c r="I18">
-        <v>173.4999999997124</v>
+        <v>173.4999999999766</v>
       </c>
       <c r="J18">
-        <v>7.414607257556509E-10</v>
+        <v>7.048912656612788E-11</v>
       </c>
       <c r="K18">
-        <v>10.00000000099686</v>
+        <v>10.00000000099975</v>
       </c>
       <c r="L18">
-        <v>1.123714967236795E-09</v>
+        <v>-4.678584044303851E-10</v>
       </c>
       <c r="M18">
         <v>3.4</v>
@@ -1592,19 +1598,19 @@
         <v>180.93</v>
       </c>
       <c r="O18">
-        <v>17664.88889002092</v>
+        <v>17664.88889002421</v>
       </c>
       <c r="P18">
-        <v>2.088016186663991E-07</v>
+        <v>-8.733853597260512E-08</v>
       </c>
       <c r="Q18">
         <v>25.5</v>
       </c>
       <c r="R18">
-        <v>-1.194825953568839E-08</v>
+        <v>-1.476024974129547E-08</v>
       </c>
       <c r="S18">
-        <v>88196.94444912035</v>
+        <v>88196.9444506315</v>
       </c>
     </row>
     <row r="19" spans="1:19">
@@ -1615,34 +1621,34 @@
         <v>26</v>
       </c>
       <c r="C19">
-        <v>1.07206371837375E-08</v>
+        <v>2.993842883114979E-10</v>
       </c>
       <c r="D19">
-        <v>-3.378647070102971E-10</v>
+        <v>-3.192189718434649E-11</v>
       </c>
       <c r="E19">
-        <v>-7.393561043674675E-11</v>
+        <v>-9.779360481782977E-11</v>
       </c>
       <c r="F19">
-        <v>-6.362669034687328E-12</v>
+        <v>-9.140922538096047E-11</v>
       </c>
       <c r="G19">
-        <v>14.00000000139703</v>
+        <v>14.00000000139974</v>
       </c>
       <c r="H19">
-        <v>4.035472735001631E-09</v>
+        <v>-1.9962018030431E-10</v>
       </c>
       <c r="I19">
-        <v>117.9409237868731</v>
+        <v>117.9409237869645</v>
       </c>
       <c r="J19">
-        <v>0.7690432943223835</v>
+        <v>0.3089731075009358</v>
       </c>
       <c r="K19">
-        <v>14.00000000139703</v>
+        <v>14.00000000139974</v>
       </c>
       <c r="L19">
-        <v>4.035472735001631E-09</v>
+        <v>-1.9962018030431E-10</v>
       </c>
       <c r="M19">
         <v>3.4</v>
@@ -1651,19 +1657,19 @@
         <v>119.2594254035402</v>
       </c>
       <c r="O19">
-        <v>24730.84444603091</v>
+        <v>24730.84444603399</v>
       </c>
       <c r="P19">
-        <v>4.974779114712619E-07</v>
+        <v>-2.546243746211478E-08</v>
       </c>
       <c r="Q19">
-        <v>8.040477887803126E-08</v>
+        <v>2.245382162336234E-09</v>
       </c>
       <c r="R19">
-        <v>-1.109034156551201E-08</v>
+        <v>-1.466904072267447E-08</v>
       </c>
       <c r="S19">
-        <v>123654.2222273206</v>
+        <v>111997.4388395918</v>
       </c>
     </row>
     <row r="20" spans="1:19">
@@ -1674,34 +1680,34 @@
         <v>27</v>
       </c>
       <c r="C20">
-        <v>1.038277247674118E-08</v>
+        <v>2.674623911271448E-10</v>
       </c>
       <c r="D20">
-        <v>-6.904143191558813E-11</v>
+        <v>-7.898009983870361E-12</v>
       </c>
       <c r="E20">
-        <v>-6.500279769010325E-11</v>
+        <v>-9.675849467574851E-11</v>
       </c>
       <c r="F20">
-        <v>-5.119451130698563E-11</v>
+        <v>-9.517889267897444E-11</v>
       </c>
       <c r="G20">
-        <v>20.00000000199707</v>
+        <v>20.00000000199972</v>
       </c>
       <c r="H20">
-        <v>7.502210741669358E-09</v>
+        <v>7.628577977216693E-11</v>
       </c>
       <c r="I20">
-        <v>106.5309659999983</v>
+        <v>106.3142919039028</v>
       </c>
       <c r="J20">
-        <v>1.14136883362298</v>
+        <v>1.599793488646659</v>
       </c>
       <c r="K20">
-        <v>20.00000000199706</v>
+        <v>20.00000000199972</v>
       </c>
       <c r="L20">
-        <v>7.502210741669358E-09</v>
+        <v>7.628577977216693E-11</v>
       </c>
       <c r="M20">
         <v>3.4</v>
@@ -1710,19 +1716,19 @@
         <v>106.0891746304491</v>
       </c>
       <c r="O20">
-        <v>35329.77778004565</v>
+        <v>35329.77778004866</v>
       </c>
       <c r="P20">
-        <v>8.198755848887201E-07</v>
+        <v>7.214776224155579E-09</v>
       </c>
       <c r="Q20">
-        <v>7.787079357555885E-08</v>
+        <v>2.005967933453586E-09</v>
       </c>
       <c r="R20">
-        <v>-9.750419653515488E-09</v>
+        <v>-1.451377420136228E-08</v>
       </c>
       <c r="S20">
-        <v>176648.8888957883</v>
+        <v>144913.6156841714</v>
       </c>
     </row>
     <row r="21" spans="1:19">
@@ -1733,34 +1739,34 @@
         <v>28</v>
       </c>
       <c r="C21">
-        <v>1.031373104482718E-08</v>
+        <v>2.595643811431048E-10</v>
       </c>
       <c r="D21">
-        <v>1.471352103167931E-11</v>
+        <v>-1.821139613762087E-12</v>
       </c>
       <c r="E21">
-        <v>-5.77003004479696E-11</v>
+        <v>-9.58867533963167E-11</v>
       </c>
       <c r="F21">
-        <v>-6.064300465430546E-11</v>
+        <v>-9.552252547356429E-11</v>
       </c>
       <c r="G21">
-        <v>28.00000000279709</v>
+        <v>28.00000000279969</v>
       </c>
       <c r="H21">
-        <v>9.65527657178415E-09</v>
+        <v>2.990840793344643E-10</v>
       </c>
       <c r="I21">
-        <v>98.88012419945412</v>
+        <v>100.3510133105022</v>
       </c>
       <c r="J21">
-        <v>3.494827411369573</v>
+        <v>5.743495166701865</v>
       </c>
       <c r="K21">
-        <v>28.00000000279709</v>
+        <v>28.00000000279969</v>
       </c>
       <c r="L21">
-        <v>9.65527657178415E-09</v>
+        <v>2.990840793344643E-10</v>
       </c>
       <c r="M21">
         <v>3.4</v>
@@ -1769,19 +1775,19 @@
         <v>95.83213549134676</v>
       </c>
       <c r="O21">
-        <v>49461.68889206526</v>
+        <v>49461.68889206821</v>
       </c>
       <c r="P21">
-        <v>9.525067354293889E-07</v>
+        <v>2.834186787077584E-08</v>
       </c>
       <c r="Q21">
-        <v>7.735298283620385E-08</v>
+        <v>1.946732858573286E-09</v>
       </c>
       <c r="R21">
-        <v>-8.65504506719544E-09</v>
+        <v>-1.438301300944751E-08</v>
       </c>
       <c r="S21">
-        <v>247308.4444552203</v>
+        <v>183753.8170845218</v>
       </c>
     </row>
     <row r="22" spans="1:19">
@@ -1795,31 +1801,31 @@
         <v>293</v>
       </c>
       <c r="D22">
-        <v>-292.9999999949853</v>
+        <v>-292.9999999999279</v>
       </c>
       <c r="E22">
-        <v>-7.579303175184762E-11</v>
+        <v>-9.808208841306117E-11</v>
       </c>
       <c r="F22">
-        <v>58.59999999892127</v>
+        <v>58.59999999988749</v>
       </c>
       <c r="G22">
-        <v>45.00000000449619</v>
+        <v>45.0000000044997</v>
       </c>
       <c r="H22">
-        <v>-5.047528441656784E-10</v>
+        <v>-5.924403512508867E-10</v>
       </c>
       <c r="I22">
-        <v>177.5964523095469</v>
+        <v>177.5964523096012</v>
       </c>
       <c r="J22">
-        <v>1.027578115602891E-11</v>
+        <v>8.158200483951862E-13</v>
       </c>
       <c r="K22">
-        <v>45.00000000449618</v>
+        <v>45.0000000044997</v>
       </c>
       <c r="L22">
-        <v>-5.047528441656784E-10</v>
+        <v>-5.924403512508867E-10</v>
       </c>
       <c r="M22">
         <v>293</v>
@@ -1828,19 +1834,19 @@
         <v>353.38</v>
       </c>
       <c r="O22">
-        <v>67866.40000435915</v>
+        <v>67866.40000436256</v>
       </c>
       <c r="P22">
-        <v>-1.841391785975893E-07</v>
+        <v>-2.161011394809002E-07</v>
       </c>
       <c r="Q22">
         <v>1831.25</v>
       </c>
       <c r="R22">
-        <v>-9.474128968980953E-09</v>
+        <v>-1.226026105163265E-08</v>
       </c>
       <c r="S22">
-        <v>330175.7500227639</v>
+        <v>330175.7500229546</v>
       </c>
     </row>
     <row r="23" spans="1:19">
@@ -1851,34 +1857,34 @@
         <v>26</v>
       </c>
       <c r="C23">
-        <v>5.01471233190897E-09</v>
+        <v>7.217734890460611E-11</v>
       </c>
       <c r="D23">
-        <v>-5.025014844287877E-10</v>
+        <v>-4.647654530676308E-11</v>
       </c>
       <c r="E23">
-        <v>-7.042683282273551E-11</v>
+        <v>-9.744511723695959E-11</v>
       </c>
       <c r="F23">
-        <v>3.007346406302203E-11</v>
+        <v>-8.814980817560697E-11</v>
       </c>
       <c r="G23">
-        <v>70.00000000699643</v>
+        <v>70.00000000699968</v>
       </c>
       <c r="H23">
-        <v>-4.558511835266582E-10</v>
+        <v>-5.87309749734832E-10</v>
       </c>
       <c r="I23">
-        <v>122.0373760966414</v>
+        <v>122.0373760965856</v>
       </c>
       <c r="J23">
-        <v>0.5818301859060708</v>
+        <v>0.6960396708178904</v>
       </c>
       <c r="K23">
-        <v>70.00000000699644</v>
+        <v>70.00000000699966</v>
       </c>
       <c r="L23">
-        <v>-4.558511835266582E-10</v>
+        <v>-5.87309749734832E-10</v>
       </c>
       <c r="M23">
         <v>293</v>
@@ -1887,19 +1893,19 @@
         <v>232.9292861830709</v>
       </c>
       <c r="O23">
-        <v>105569.9555623387</v>
+        <v>105569.9555623419</v>
       </c>
       <c r="P23">
-        <v>-1.114274302253982E-07</v>
+        <v>-1.434909880445296E-07</v>
       </c>
       <c r="Q23">
-        <v>3.134195207443106E-08</v>
+        <v>4.511084306537882E-10</v>
       </c>
       <c r="R23">
-        <v>-8.803354102841939E-09</v>
+        <v>-1.218063965461995E-08</v>
       </c>
       <c r="S23">
-        <v>527849.7778121381</v>
+        <v>478089.8067266438</v>
       </c>
     </row>
     <row r="24" spans="1:19">
@@ -1910,34 +1916,34 @@
         <v>27</v>
       </c>
       <c r="C24">
-        <v>4.512210847475683E-09</v>
+        <v>2.570080359789184E-11</v>
       </c>
       <c r="D24">
-        <v>-1.473609083706961E-10</v>
+        <v>-1.53922587106765E-11</v>
       </c>
       <c r="E24">
-        <v>-6.24173516375172E-11</v>
+        <v>-9.64448522187623E-11</v>
       </c>
       <c r="F24">
-        <v>-3.294516996337799E-11</v>
+        <v>-9.3366400476627E-11</v>
       </c>
       <c r="G24">
-        <v>79.00000000789649</v>
+        <v>79.00000000789966</v>
       </c>
       <c r="H24">
-        <v>-4.375961951274701E-10</v>
+        <v>-5.841781402594422E-10</v>
       </c>
       <c r="I24">
-        <v>110.6274183097069</v>
+        <v>110.4107442135196</v>
       </c>
       <c r="J24">
-        <v>0.6479505948924282</v>
+        <v>0.892089782547575</v>
       </c>
       <c r="K24">
-        <v>79.00000000789649</v>
+        <v>79.00000000789964</v>
       </c>
       <c r="L24">
-        <v>-4.375961951274701E-10</v>
+        <v>-5.841781402594422E-10</v>
       </c>
       <c r="M24">
         <v>293</v>
@@ -1946,19 +1952,19 @@
         <v>207.2060605256625</v>
       </c>
       <c r="O24">
-        <v>119143.2355632114</v>
+        <v>119143.2355632144</v>
       </c>
       <c r="P24">
-        <v>-9.572733503046435E-08</v>
+        <v>-1.277011063093278E-07</v>
       </c>
       <c r="Q24">
-        <v>2.820131779672302E-08</v>
+        <v>1.60630022486824E-10</v>
       </c>
       <c r="R24">
-        <v>-7.80216895468965E-09</v>
+        <v>-1.205560652734529E-08</v>
       </c>
       <c r="S24">
-        <v>595716.1778164335</v>
+        <v>488694.753680113</v>
       </c>
     </row>
     <row r="25" spans="1:19">
@@ -1969,34 +1975,34 @@
         <v>28</v>
       </c>
       <c r="C25">
-        <v>4.364849939101387E-09</v>
+        <v>1.030854488720624E-11</v>
       </c>
       <c r="D25">
-        <v>2.940539497913278E-11</v>
+        <v>2.455750551060589E-12</v>
       </c>
       <c r="E25">
-        <v>-4.871984634496036E-11</v>
+        <v>-9.464768254937466E-11</v>
       </c>
       <c r="F25">
-        <v>-5.460092534078692E-11</v>
+        <v>-9.513883265958678E-11</v>
       </c>
       <c r="G25">
-        <v>89.00000000889652</v>
+        <v>89.00000000889963</v>
       </c>
       <c r="H25">
-        <v>-4.161133301638424E-10</v>
+        <v>-5.799358465875039E-10</v>
       </c>
       <c r="I25">
-        <v>102.9765765091269</v>
+        <v>104.447465620116</v>
       </c>
       <c r="J25">
-        <v>0.6728768169281742</v>
+        <v>1.054029688317087</v>
       </c>
       <c r="K25">
-        <v>89.00000000889652</v>
+        <v>89.00000000889963</v>
       </c>
       <c r="L25">
-        <v>-4.161133301638424E-10</v>
+        <v>-5.799358465875039E-10</v>
       </c>
       <c r="M25">
         <v>293</v>
@@ -2005,19 +2011,19 @@
         <v>187.1727189517057</v>
       </c>
       <c r="O25">
-        <v>134224.6577864031</v>
+        <v>134224.6577864062</v>
       </c>
       <c r="P25">
-        <v>-8.271701528840204E-08</v>
+        <v>-1.151591684464517E-07</v>
       </c>
       <c r="Q25">
-        <v>2.728031211938367E-08</v>
+        <v>6.442840554503901E-11</v>
       </c>
       <c r="R25">
-        <v>-6.089980793120045E-09</v>
+        <v>-1.183096031867183E-08</v>
       </c>
       <c r="S25">
-        <v>671123.2889323233</v>
+        <v>498654.4893153113</v>
       </c>
     </row>
   </sheetData>
@@ -2061,7 +2067,7 @@
         <v>25</v>
       </c>
       <c r="D2">
-        <v>324.0000000326239</v>
+        <v>324.0000000328782</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -2081,7 +2087,7 @@
         <v>26</v>
       </c>
       <c r="D3">
-        <v>350.0000000351367</v>
+        <v>350.0000000354681</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -2101,7 +2107,7 @@
         <v>27</v>
       </c>
       <c r="D4">
-        <v>333.0000000334107</v>
+        <v>333.0000000337623</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -2121,7 +2127,7 @@
         <v>28</v>
       </c>
       <c r="D5">
-        <v>316.0000000316977</v>
+        <v>316.0000000320568</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -2141,7 +2147,7 @@
         <v>25</v>
       </c>
       <c r="D6">
-        <v>75.00000000742021</v>
+        <v>75.00000000795517</v>
       </c>
       <c r="E6">
         <v>16.118</v>
@@ -2161,7 +2167,7 @@
         <v>26</v>
       </c>
       <c r="D7">
-        <v>90.00000000794078</v>
+        <v>90.00000000936279</v>
       </c>
       <c r="E7">
         <v>16.118</v>
@@ -2181,7 +2187,7 @@
         <v>27</v>
       </c>
       <c r="D8">
-        <v>95.00000000749905</v>
+        <v>95.0000000097796</v>
       </c>
       <c r="E8">
         <v>16.118</v>
@@ -2201,7 +2207,7 @@
         <v>28</v>
       </c>
       <c r="D9">
-        <v>99.00000000745655</v>
+        <v>99.0000000101157</v>
       </c>
       <c r="E9">
         <v>16.118</v>
@@ -2221,7 +2227,7 @@
         <v>25</v>
       </c>
       <c r="D10">
-        <v>45.0000000046216</v>
+        <v>45.0000000049703</v>
       </c>
       <c r="E10">
         <v>11.133</v>
@@ -2241,7 +2247,7 @@
         <v>26</v>
       </c>
       <c r="D11">
-        <v>65.00000000643189</v>
+        <v>65.00000000695022</v>
       </c>
       <c r="E11">
         <v>11.133</v>
@@ -2261,7 +2267,7 @@
         <v>27</v>
       </c>
       <c r="D12">
-        <v>70.00000000686659</v>
+        <v>70.00000000743869</v>
       </c>
       <c r="E12">
         <v>11.133</v>
@@ -2281,7 +2287,7 @@
         <v>28</v>
       </c>
       <c r="D13">
-        <v>75.00000000734003</v>
+        <v>75.0000000079294</v>
       </c>
       <c r="E13">
         <v>11.133</v>
@@ -2301,7 +2307,7 @@
         <v>25</v>
       </c>
       <c r="D14">
-        <v>50.00000000487391</v>
+        <v>50.00000000545097</v>
       </c>
       <c r="E14">
         <v>13.78042157888167</v>
@@ -2321,7 +2327,7 @@
         <v>26</v>
       </c>
       <c r="D15">
-        <v>85.00000000706859</v>
+        <v>85.00000000883088</v>
       </c>
       <c r="E15">
         <v>13.78042157888167</v>
@@ -2341,7 +2347,7 @@
         <v>27</v>
       </c>
       <c r="D16">
-        <v>103.000000008931</v>
+        <v>103.0000000098062</v>
       </c>
       <c r="E16">
         <v>13.78042157888167</v>
@@ -2361,7 +2367,7 @@
         <v>28</v>
       </c>
       <c r="D17">
-        <v>93.00000002115303</v>
+        <v>93.00000001015729</v>
       </c>
       <c r="E17">
         <v>13.78042157888167</v>
@@ -2381,7 +2387,7 @@
         <v>25</v>
       </c>
       <c r="D18">
-        <v>10.00000000089922</v>
+        <v>10.00000000145415</v>
       </c>
       <c r="E18">
         <v>10.5</v>
@@ -2401,7 +2407,7 @@
         <v>26</v>
       </c>
       <c r="D19">
-        <v>13.99999999991183</v>
+        <v>14.00000000173175</v>
       </c>
       <c r="E19">
         <v>10.5</v>
@@ -2421,7 +2427,7 @@
         <v>27</v>
       </c>
       <c r="D20">
-        <v>19.99999999821381</v>
+        <v>20.00000000216881</v>
       </c>
       <c r="E20">
         <v>10.5</v>
@@ -2441,7 +2447,7 @@
         <v>28</v>
       </c>
       <c r="D21">
-        <v>27.99999999735236</v>
+        <v>28.00000000282657</v>
       </c>
       <c r="E21">
         <v>10.5</v>
@@ -2461,7 +2467,7 @@
         <v>25</v>
       </c>
       <c r="D22">
-        <v>45.00000000454443</v>
+        <v>45.00000000496451</v>
       </c>
       <c r="E22">
         <v>14.59645230960589</v>
@@ -2481,7 +2487,7 @@
         <v>26</v>
       </c>
       <c r="D23">
-        <v>70.00000000667377</v>
+        <v>70.00000000742763</v>
       </c>
       <c r="E23">
         <v>14.59645230960589</v>
@@ -2501,7 +2507,7 @@
         <v>27</v>
       </c>
       <c r="D24">
-        <v>79.0000000074108</v>
+        <v>79.00000000830529</v>
       </c>
       <c r="E24">
         <v>14.59645230960589</v>
@@ -2521,7 +2527,7 @@
         <v>28</v>
       </c>
       <c r="D25">
-        <v>89.00000000835144</v>
+        <v>89.00000000928921</v>
       </c>
       <c r="E25">
         <v>14.59645230960589</v>
@@ -2541,7 +2547,7 @@
         <v>28</v>
       </c>
       <c r="D26">
-        <v>32.9999999910362</v>
+        <v>33.00000000275709</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -2582,10 +2588,10 @@
         <v>35</v>
       </c>
       <c r="C2">
-        <v>700.0000000745171</v>
+        <v>700.0000000723545</v>
       </c>
       <c r="D2">
-        <v>17500.00000186293</v>
+        <v>11776.99833060832</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2596,10 +2602,10 @@
         <v>35</v>
       </c>
       <c r="C3">
-        <v>3.091685888569995E-09</v>
+        <v>-8.848614266095167E-11</v>
       </c>
       <c r="D3">
-        <v>2.705225152498745E-07</v>
+        <v>-5.21050577146141E-09</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2610,10 +2616,10 @@
         <v>35</v>
       </c>
       <c r="C4">
-        <v>3.072760523104142E-09</v>
+        <v>-8.554518189924889E-11</v>
       </c>
       <c r="D4">
-        <v>2.688665457716125E-07</v>
+        <v>-5.037327321574519E-09</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2624,10 +2630,10 @@
         <v>35</v>
       </c>
       <c r="C5">
-        <v>32.99999999224631</v>
+        <v>33.0000000023129</v>
       </c>
       <c r="D5">
-        <v>948.7499997770814</v>
+        <v>638.4815523310194</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2638,10 +2644,10 @@
         <v>35</v>
       </c>
       <c r="C6">
-        <v>1.032844456586458E-08</v>
+        <v>2.577432415294817E-10</v>
       </c>
       <c r="D6">
-        <v>7.746333424398432E-07</v>
+        <v>1.300903596387655E-08</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2652,10 +2658,10 @@
         <v>35</v>
       </c>
       <c r="C7">
-        <v>4.394255334090472E-09</v>
+        <v>1.276429543824201E-11</v>
       </c>
       <c r="D7">
-        <v>2.746409583806545E-07</v>
+        <v>5.368753073286766E-10</v>
       </c>
     </row>
   </sheetData>
@@ -2665,7 +2671,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2681,7 +2687,7 @@
         <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -2689,7 +2695,7 @@
         <v>39</v>
       </c>
       <c r="B3">
-        <v>11874785.71906545</v>
+        <v>10127116.53173693</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -2697,7 +2703,7 @@
         <v>40</v>
       </c>
       <c r="B4">
-        <v>11856336.96906222</v>
+        <v>10114701.05185399</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -2705,7 +2711,7 @@
         <v>41</v>
       </c>
       <c r="B5">
-        <v>18448.75000322867</v>
+        <v>12415.47988294264</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -2720,16 +2726,16 @@
       <c r="A7" t="s">
         <v>43</v>
       </c>
-      <c r="B7" t="s">
-        <v>50</v>
+      <c r="B7">
+        <v>0.02</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>44</v>
       </c>
-      <c r="B8" t="s">
-        <v>51</v>
+      <c r="B8">
+        <v>2025</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -2762,6 +2768,22 @@
       </c>
       <c r="B12" t="s">
         <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>